<commit_message>
updated the downloaded excel file with full data
</commit_message>
<xml_diff>
--- a/For Research paper/linear_regression_summary.xlsx
+++ b/For Research paper/linear_regression_summary.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,7 +437,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>0.702</t>
+          <t>0.695</t>
         </is>
       </c>
     </row>
@@ -459,7 +459,7 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>-6844.4151</t>
+          <t>-6755.1027</t>
         </is>
       </c>
     </row>
@@ -471,7 +471,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2024-09-30 16:21</t>
+          <t>2025-01-07 21:06</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
@@ -481,7 +481,7 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>-6619.9994</t>
+          <t>-6549.3884</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>3458.2</t>
+          <t>3410.6</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
@@ -525,7 +525,7 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>255.0</t>
+          <t>269.2</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>3730</t>
+          <t>3733</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
@@ -559,7 +559,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>0.705</t>
+          <t>0.698</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
@@ -569,895 +569,755 @@
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>0.0094210</t>
+          <t>0.0096547</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>5.385480194416095</v>
+        <v>7.959617672140032</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.00497286539007933</v>
+        <v>0.01283511423654921</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>1082.973250223084</v>
+        <v>620.1438900694986</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>5.375730393611791</v>
+        <v>7.934453151356387</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>5.395229995220399</v>
+        <v>7.984782192923678</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>-9.33360368353606e-08</v>
+        <v>-7.889797709761638e-08</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>3.648059838067716e-08</v>
+        <v>3.679300389493554e-08</v>
       </c>
       <c r="C11" s="1" t="n">
-        <v>-2.558511674106703</v>
+        <v>-2.144374439306829</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>0.01055128135933388</v>
+        <v>0.03206727896621936</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>-1.648599047733437e-07</v>
+        <v>-1.510343285272238e-07</v>
       </c>
       <c r="F11" s="1" t="n">
-        <v>-2.181216889737749e-08</v>
+        <v>-6.761625668008928e-09</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>-0.01836011510207283</v>
+        <v>-0.01798934237141374</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.0003261491125836136</v>
+        <v>0.0003258531214769697</v>
       </c>
       <c r="C12" s="1" t="n">
-        <v>-56.29362274400155</v>
+        <v>-55.2069051536926</v>
       </c>
       <c r="D12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>-0.01899956311257687</v>
+        <v>-0.01862820989504458</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>-0.0177206670915688</v>
+        <v>-0.0173504748477829</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>-0.02374704222780089</v>
+        <v>0.08818921220976705</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.005519325699795688</v>
+        <v>0.0154357961522593</v>
       </c>
       <c r="C13" s="1" t="n">
-        <v>-4.302525982237277</v>
+        <v>5.713292099731377</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>1.731922598763204e-05</v>
+        <v>1.194705369436427e-08</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>-0.03456823321648815</v>
+        <v>0.05792579531087048</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>-0.01292585123911362</v>
+        <v>0.1184526291086636</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>-0.009968022628430551</v>
+        <v>0.06398367005534472</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.004102141426126016</v>
+        <v>0.00692595306973034</v>
       </c>
       <c r="C14" s="1" t="n">
-        <v>-2.429955867670843</v>
+        <v>9.238247705573308</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>0.01514753918317543</v>
+        <v>4.097126230903009e-20</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>-0.01801068186782981</v>
+        <v>0.05040464872700445</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>-0.001925363389031289</v>
+        <v>0.07756269138368499</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>0.03844595826708852</v>
+        <v>0.05540672690985946</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.005128918506643284</v>
+        <v>0.009126094677605877</v>
       </c>
       <c r="C15" s="1" t="n">
-        <v>7.495919113803621</v>
+        <v>6.071241737807036</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>8.178391510002915e-14</v>
+        <v>1.396094683965651e-09</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>0.0283901996935631</v>
+        <v>0.03751410866309912</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>0.04850171684061394</v>
+        <v>0.07329934515661979</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>0.4144667218445335</v>
+        <v>-0.08880445573639795</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.006048725037118981</v>
+        <v>0.01040057024085314</v>
       </c>
       <c r="C16" s="1" t="n">
-        <v>68.52133619913144</v>
+        <v>-8.538421805717597</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>0</v>
+        <v>1.952237137879361e-17</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>0.4026075904170945</v>
+        <v>-0.1091958103565563</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>0.4263258532719726</v>
+        <v>-0.06841310111623958</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>0.5021543625941804</v>
+        <v>0.0567863115006165</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.013040474841852</v>
+        <v>0.007284507416228288</v>
       </c>
       <c r="C17" s="1" t="n">
-        <v>38.50736792057372</v>
+        <v>7.795490931083278</v>
       </c>
       <c r="D17" s="1" t="n">
-        <v>1.929723626541019e-273</v>
+        <v>8.260238046143919e-15</v>
       </c>
       <c r="E17" s="1" t="n">
-        <v>0.4765872052053575</v>
+        <v>0.04250430863754077</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>0.5277215199830034</v>
+        <v>0.07106831436369222</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>0.4772253815130125</v>
+        <v>0.04700066804339045</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.003984133435622555</v>
+        <v>0.0103127246588845</v>
       </c>
       <c r="C18" s="1" t="n">
-        <v>119.7814755013199</v>
+        <v>4.557541251030975</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>0</v>
+        <v>5.341290418367887e-06</v>
       </c>
       <c r="E18" s="1" t="n">
-        <v>0.4694140887616385</v>
+        <v>0.0267815434425728</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>0.4850366742643866</v>
+        <v>0.0672197926442081</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>0.4653795304907724</v>
+        <v>0.0504485737779167</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.006521917850662272</v>
+        <v>0.008947716221494817</v>
       </c>
       <c r="C19" s="1" t="n">
-        <v>71.35623924541079</v>
+        <v>5.638150845321366</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>0</v>
+        <v>1.846220302504101e-08</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>0.4525926571455089</v>
+        <v>0.03290568427399678</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>0.4781664038360358</v>
+        <v>0.06799146328183661</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>0.3223291668821038</v>
+        <v>0.02071955739368072</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.007823316244846574</v>
+        <v>0.01138555735833902</v>
       </c>
       <c r="C20" s="1" t="n">
-        <v>41.20109130120242</v>
+        <v>1.819810549591169</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>3.73260755270039e-306</v>
+        <v>0.06886791465122073</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>0.3069907716043041</v>
+        <v>-0.001602962647585832</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>0.3376675621599035</v>
+        <v>0.04304207743494726</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>0.4671374422246116</v>
+        <v>-0.108038693753161</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.004385660286778291</v>
+        <v>0.008690197311816332</v>
       </c>
       <c r="C21" s="1" t="n">
-        <v>106.5147347670585</v>
+        <v>-12.43224864483312</v>
       </c>
       <c r="D21" s="1" t="n">
-        <v>0</v>
+        <v>8.455907975613571e-35</v>
       </c>
       <c r="E21" s="1" t="n">
-        <v>0.458538915854536</v>
+        <v>-0.1250766917668024</v>
       </c>
       <c r="F21" s="1" t="n">
-        <v>0.4757359685946871</v>
+        <v>-0.09100069573951959</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>0.4595895738156573</v>
+        <v>0.1638056421796415</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.00768404072227853</v>
+        <v>0.009415927198328674</v>
       </c>
       <c r="C22" s="1" t="n">
-        <v>59.81092376087464</v>
+        <v>17.39665555280811</v>
       </c>
       <c r="D22" s="1" t="n">
-        <v>0</v>
+        <v>3.068541971488e-65</v>
       </c>
       <c r="E22" s="1" t="n">
-        <v>0.4445242421531855</v>
+        <v>0.1453447783873342</v>
       </c>
       <c r="F22" s="1" t="n">
-        <v>0.4746549054781291</v>
+        <v>0.1822665059719488</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>0.4599693899354363</v>
+        <v>0.09795746148125282</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.006148196332176788</v>
+        <v>0.01066201216913145</v>
       </c>
       <c r="C23" s="1" t="n">
-        <v>74.81371203586512</v>
+        <v>9.187521072697544</v>
       </c>
       <c r="D23" s="1" t="n">
-        <v>0</v>
+        <v>6.504509492964021e-20</v>
       </c>
       <c r="E23" s="1" t="n">
-        <v>0.4479152350684941</v>
+        <v>0.07705352390182935</v>
       </c>
       <c r="F23" s="1" t="n">
-        <v>0.4720235448023786</v>
+        <v>0.1188613990606763</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>0.4300060618062246</v>
+        <v>0.001509196454297465</v>
       </c>
       <c r="B24" s="1" t="n">
-        <v>0.009124497120768521</v>
+        <v>0.01101950841216781</v>
       </c>
       <c r="C24" s="1" t="n">
-        <v>47.12654912537326</v>
+        <v>0.1369567858971822</v>
       </c>
       <c r="D24" s="1" t="n">
-        <v>0</v>
+        <v>0.8910723386616416</v>
       </c>
       <c r="E24" s="1" t="n">
-        <v>0.4121165710622342</v>
+        <v>-0.02009564814255998</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>0.447895552550215</v>
+        <v>0.02311404105115491</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>0.3021265506429884</v>
+        <v>0.01282205861526758</v>
       </c>
       <c r="B25" s="1" t="n">
-        <v>0.006183887554546755</v>
+        <v>0.01380698831338865</v>
       </c>
       <c r="C25" s="1" t="n">
-        <v>48.85705763211158</v>
+        <v>0.9286644070549421</v>
       </c>
       <c r="D25" s="1" t="n">
-        <v>0</v>
+        <v>0.353123074494291</v>
       </c>
       <c r="E25" s="1" t="n">
-        <v>0.2900024195588609</v>
+        <v>-0.01424791816627434</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>0.3142506817271159</v>
+        <v>0.03989203539680951</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>0.5736949839056718</v>
+        <v>-0.01210559690259067</v>
       </c>
       <c r="B26" s="1" t="n">
-        <v>0.006706177111158554</v>
+        <v>0.01600759450064856</v>
       </c>
       <c r="C26" s="1" t="n">
-        <v>85.54724612791514</v>
+        <v>-0.7562408519343865</v>
       </c>
       <c r="D26" s="1" t="n">
-        <v>0</v>
+        <v>0.4495525233329695</v>
       </c>
       <c r="E26" s="1" t="n">
-        <v>0.5605468518201715</v>
+        <v>-0.04349008145674204</v>
       </c>
       <c r="F26" s="1" t="n">
-        <v>0.586843115991172</v>
+        <v>0.01927888765156071</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>0.5114010287609216</v>
+        <v>0.01088534962043988</v>
       </c>
       <c r="B27" s="1" t="n">
-        <v>0.008089079151371003</v>
+        <v>0.01018551497716373</v>
       </c>
       <c r="C27" s="1" t="n">
-        <v>63.22116760030036</v>
+        <v>1.068708812941241</v>
       </c>
       <c r="D27" s="1" t="n">
-        <v>0</v>
+        <v>0.2852700005133898</v>
       </c>
       <c r="E27" s="1" t="n">
-        <v>0.4955415786793955</v>
+        <v>-0.009084367719908854</v>
       </c>
       <c r="F27" s="1" t="n">
-        <v>0.5272604788424478</v>
+        <v>0.03085506696078862</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>0.5371724970347749</v>
+        <v>0.003993778592552455</v>
       </c>
       <c r="B28" s="1" t="n">
-        <v>0.008642153771933343</v>
+        <v>0.01635065934441098</v>
       </c>
       <c r="C28" s="1" t="n">
-        <v>62.1572482058027</v>
+        <v>0.2442579536658024</v>
       </c>
       <c r="D28" s="1" t="n">
-        <v>0</v>
+        <v>0.8070444689889106</v>
       </c>
       <c r="E28" s="1" t="n">
-        <v>0.520228688749796</v>
+        <v>-0.02806331878232584</v>
       </c>
       <c r="F28" s="1" t="n">
-        <v>0.5541163053197538</v>
+        <v>0.03605087596743075</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>0.5388203447358872</v>
+        <v>0.0003194433053073931</v>
       </c>
       <c r="B29" s="1" t="n">
-        <v>0.005782727668546478</v>
+        <v>0.01076850960122609</v>
       </c>
       <c r="C29" s="1" t="n">
-        <v>93.17754105327302</v>
+        <v>0.02966457914204039</v>
       </c>
       <c r="D29" s="1" t="n">
-        <v>0</v>
+        <v>0.9763361469884868</v>
       </c>
       <c r="E29" s="1" t="n">
-        <v>0.5274827277985096</v>
+        <v>-0.02079329310472711</v>
       </c>
       <c r="F29" s="1" t="n">
-        <v>0.5501579616732649</v>
+        <v>0.0214321797153419</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>0.5433154650043068</v>
+        <v>0.001514062580567715</v>
       </c>
       <c r="B30" s="1" t="n">
-        <v>0.009415303854244347</v>
+        <v>0.01063183866131455</v>
       </c>
       <c r="C30" s="1" t="n">
-        <v>57.70556887119308</v>
+        <v>0.1424083480571282</v>
       </c>
       <c r="D30" s="1" t="n">
-        <v>0</v>
+        <v>0.8867651540535382</v>
       </c>
       <c r="E30" s="1" t="n">
-        <v>0.5248558185248333</v>
+        <v>-0.0193307168292766</v>
       </c>
       <c r="F30" s="1" t="n">
-        <v>0.5617751114837803</v>
+        <v>0.02235884199041203</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>0.5271050653434762</v>
+        <v>0.007113186383080061</v>
       </c>
       <c r="B31" s="1" t="n">
-        <v>0.01203618185197014</v>
+        <v>0.009864747448957359</v>
       </c>
       <c r="C31" s="1" t="n">
-        <v>43.79337831765952</v>
+        <v>0.721071311747761</v>
       </c>
       <c r="D31" s="1" t="n">
-        <v>0</v>
+        <v>0.4709107951557275</v>
       </c>
       <c r="E31" s="1" t="n">
-        <v>0.5035069249765176</v>
+        <v>-0.01222763424614457</v>
       </c>
       <c r="F31" s="1" t="n">
-        <v>0.5507032057104349</v>
+        <v>0.0264540070123047</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>0.5486245768032946</v>
+        <v>0.00163885131994429</v>
       </c>
       <c r="B32" s="1" t="n">
-        <v>0.004356344693146157</v>
+        <v>0.01011339293867119</v>
       </c>
       <c r="C32" s="1" t="n">
-        <v>125.9369070740537</v>
+        <v>0.1620476263389031</v>
       </c>
       <c r="D32" s="1" t="n">
-        <v>0</v>
+        <v>0.8712771191847407</v>
       </c>
       <c r="E32" s="1" t="n">
-        <v>0.5400835265915207</v>
+        <v>-0.01818946357527183</v>
       </c>
       <c r="F32" s="1" t="n">
-        <v>0.5571656270150684</v>
+        <v>0.02146716621516041</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>0.5319432744204275</v>
+        <v>0.0163641699385314</v>
       </c>
       <c r="B33" s="1" t="n">
-        <v>0.01234990124510475</v>
+        <v>0.01336673089754567</v>
       </c>
       <c r="C33" s="1" t="n">
-        <v>43.07267433666964</v>
+        <v>1.224246232228413</v>
       </c>
       <c r="D33" s="1" t="n">
-        <v>0</v>
+        <v>0.2209366093191774</v>
       </c>
       <c r="E33" s="1" t="n">
-        <v>0.5077300557532175</v>
+        <v>-0.009842638297179681</v>
       </c>
       <c r="F33" s="1" t="n">
-        <v>0.5561564930876376</v>
+        <v>0.04257097817424249</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>0.5335672155453318</v>
+        <v>-0.04394877823658658</v>
       </c>
       <c r="B34" s="1" t="n">
-        <v>0.00534394922556819</v>
+        <v>0.008720348372103802</v>
       </c>
       <c r="C34" s="1" t="n">
-        <v>99.84511323432361</v>
+        <v>-5.039796159655471</v>
       </c>
       <c r="D34" s="1" t="n">
-        <v>0</v>
+        <v>4.881366418879702e-07</v>
       </c>
       <c r="E34" s="1" t="n">
-        <v>0.5230898677044784</v>
+        <v>-0.0610458904091883</v>
       </c>
       <c r="F34" s="1" t="n">
-        <v>0.5440445633861852</v>
+        <v>-0.02685166606398485</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>0.5397903873287557</v>
+        <v>0.09303633073543768</v>
       </c>
       <c r="B35" s="1" t="n">
-        <v>0.005216593112937004</v>
+        <v>0.004597496394980953</v>
       </c>
       <c r="C35" s="1" t="n">
-        <v>103.4756546356071</v>
+        <v>20.23630314033626</v>
       </c>
       <c r="D35" s="1" t="n">
-        <v>0</v>
+        <v>1.743895249853198e-86</v>
       </c>
       <c r="E35" s="1" t="n">
-        <v>0.5295627339059016</v>
+        <v>0.08402248080375679</v>
       </c>
       <c r="F35" s="1" t="n">
-        <v>0.5500180407516099</v>
+        <v>0.1020501806671186</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>0.5449697946418307</v>
+        <v>-0.0063936423268523</v>
       </c>
       <c r="B36" s="1" t="n">
-        <v>0.003709411835651714</v>
+        <v>0.00590862073596374</v>
       </c>
       <c r="C36" s="1" t="n">
-        <v>146.9154191519109</v>
+        <v>-1.082087108406942</v>
       </c>
       <c r="D36" s="1" t="n">
-        <v>0</v>
+        <v>0.2792837168939903</v>
       </c>
       <c r="E36" s="1" t="n">
-        <v>0.5376971211102125</v>
+        <v>-0.01797808221359977</v>
       </c>
       <c r="F36" s="1" t="n">
-        <v>0.5522424681734489</v>
+        <v>0.005190797559895167</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>0.5401715735580307</v>
+        <v>-0.1184478052970424</v>
       </c>
       <c r="B37" s="1" t="n">
-        <v>0.004204150533960132</v>
+        <v>0.009582647230057823</v>
       </c>
       <c r="C37" s="1" t="n">
-        <v>128.4853073634383</v>
+        <v>-12.36065592871956</v>
       </c>
       <c r="D37" s="1" t="n">
-        <v>0</v>
+        <v>1.99403425128606e-34</v>
       </c>
       <c r="E37" s="1" t="n">
-        <v>0.5319289152429292</v>
+        <v>-0.1372355403291514</v>
       </c>
       <c r="F37" s="1" t="n">
-        <v>0.5484142318731322</v>
+        <v>-0.09966007026493329</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>0.915153892086165</v>
+        <v>0.07891285745813462</v>
       </c>
       <c r="B38" s="1" t="n">
-        <v>0.004198868089570255</v>
+        <v>0.005010677002544422</v>
       </c>
       <c r="C38" s="1" t="n">
-        <v>217.9525225761091</v>
+        <v>15.74894119458562</v>
       </c>
       <c r="D38" s="1" t="n">
-        <v>0</v>
+        <v>3.73077474066547e-54</v>
       </c>
       <c r="E38" s="1" t="n">
-        <v>0.9069215905325122</v>
+        <v>0.06908892576209962</v>
       </c>
       <c r="F38" s="1" t="n">
-        <v>0.9233861936398179</v>
+        <v>0.08873678915416962</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>0.9251133620108507</v>
+        <v>0.1509211784452207</v>
       </c>
       <c r="B39" s="1" t="n">
-        <v>0.01126037978494656</v>
+        <v>0.006964659862561015</v>
       </c>
       <c r="C39" s="1" t="n">
-        <v>82.15649735434224</v>
+        <v>21.6695691424225</v>
       </c>
       <c r="D39" s="1" t="n">
-        <v>0</v>
+        <v>3.518833980610106e-98</v>
       </c>
       <c r="E39" s="1" t="n">
-        <v>0.9030362593201052</v>
+        <v>0.1372662685914879</v>
       </c>
       <c r="F39" s="1" t="n">
-        <v>0.9471904647015962</v>
+        <v>0.1645760882989534</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>0.8473146735040602</v>
+        <v>0.2581457508543119</v>
       </c>
       <c r="B40" s="1" t="n">
-        <v>0.007104705057607198</v>
+        <v>0.008789873083347319</v>
       </c>
       <c r="C40" s="1" t="n">
-        <v>119.2610624415461</v>
+        <v>29.36854132096364</v>
       </c>
       <c r="D40" s="1" t="n">
-        <v>0</v>
+        <v>9.523747843326642e-171</v>
       </c>
       <c r="E40" s="1" t="n">
-        <v>0.8333851874529823</v>
+        <v>0.2409123285555343</v>
       </c>
       <c r="F40" s="1" t="n">
-        <v>0.8612441595551381</v>
+        <v>0.2753791731530894</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>0.9924679704450337</v>
+        <v>0.2408961381460534</v>
       </c>
       <c r="B41" s="1" t="n">
-        <v>0.003761641400885278</v>
+        <v>0.01171265549670269</v>
       </c>
       <c r="C41" s="1" t="n">
-        <v>263.8390704152349</v>
+        <v>20.56716670390158</v>
       </c>
       <c r="D41" s="1" t="n">
-        <v>0</v>
+        <v>3.960431892757484e-89</v>
       </c>
       <c r="E41" s="1" t="n">
-        <v>0.9850928956181505</v>
+        <v>0.2179323096014543</v>
       </c>
       <c r="F41" s="1" t="n">
-        <v>0.9998430452719168</v>
+        <v>0.2638599666906526</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>0.9119246672160253</v>
+        <v>0.2774801315764147</v>
       </c>
       <c r="B42" s="1" t="n">
-        <v>0.00540076862659462</v>
+        <v>0.01175536163408736</v>
       </c>
       <c r="C42" s="1" t="n">
-        <v>168.8509044296954</v>
+        <v>23.60455936734413</v>
       </c>
       <c r="D42" s="1" t="n">
-        <v>0</v>
+        <v>6.165127176591511e-115</v>
       </c>
       <c r="E42" s="1" t="n">
-        <v>0.9013359192470018</v>
+        <v>0.2544325733927956</v>
       </c>
       <c r="F42" s="1" t="n">
-        <v>0.9225134151850487</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="n">
-        <v>0.7935056291539964</v>
-      </c>
-      <c r="B43" s="1" t="n">
-        <v>0.008208641829467612</v>
-      </c>
-      <c r="C43" s="1" t="n">
-        <v>96.66710347934145</v>
-      </c>
-      <c r="D43" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E43" s="1" t="n">
-        <v>0.7774117644636621</v>
-      </c>
-      <c r="F43" s="1" t="n">
-        <v>0.8095994938443306</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>0.7471059973587123</v>
-      </c>
-      <c r="B44" s="1" t="n">
-        <v>0.005573709230252089</v>
-      </c>
-      <c r="C44" s="1" t="n">
-        <v>134.0410786597352</v>
-      </c>
-      <c r="D44" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E44" s="1" t="n">
-        <v>0.7361781820101454</v>
-      </c>
-      <c r="F44" s="1" t="n">
-        <v>0.7580338127072792</v>
+        <v>0.3005276897600338</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>0.8237546132923446</v>
-      </c>
-      <c r="B45" s="1" t="n">
-        <v>0.004388315061318846</v>
-      </c>
-      <c r="C45" s="1" t="n">
-        <v>187.7154675044632</v>
-      </c>
-      <c r="D45" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E45" s="1" t="n">
-        <v>0.8151508819708134</v>
-      </c>
-      <c r="F45" s="1" t="n">
-        <v>0.8323583446138757</v>
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>Omnibus:</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
+        <is>
+          <t>1093.471</t>
+        </is>
+      </c>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>Durbin-Watson:</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>1.671</t>
+        </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>0.8854007971906609</v>
-      </c>
-      <c r="B46" s="1" t="n">
-        <v>0.005067570409383244</v>
-      </c>
-      <c r="C46" s="1" t="n">
-        <v>174.7189926658404</v>
-      </c>
-      <c r="D46" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E46" s="1" t="n">
-        <v>0.8754653177079795</v>
-      </c>
-      <c r="F46" s="1" t="n">
-        <v>0.8953362766733423</v>
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>Prob(Omnibus):</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>Jarque-Bera (JB):</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>18218.884</t>
+        </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>0.9737155894568408</v>
-      </c>
-      <c r="B47" s="1" t="n">
-        <v>0.006034266228078141</v>
-      </c>
-      <c r="C47" s="1" t="n">
-        <v>161.3643735051048</v>
-      </c>
-      <c r="D47" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E47" s="1" t="n">
-        <v>0.9618848059730837</v>
-      </c>
-      <c r="F47" s="1" t="n">
-        <v>0.9855463729405979</v>
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>Skew:</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>0.936</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>Prob(JB):</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>0.96061887870509</v>
-      </c>
-      <c r="B48" s="1" t="n">
-        <v>0.008609548860232019</v>
-      </c>
-      <c r="C48" s="1" t="n">
-        <v>111.5759831670439</v>
-      </c>
-      <c r="D48" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" s="1" t="n">
-        <v>0.9437389956160281</v>
-      </c>
-      <c r="F48" s="1" t="n">
-        <v>0.9774987617941518</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>0.9948843184124718</v>
-      </c>
-      <c r="B49" s="1" t="n">
-        <v>0.008889723928998372</v>
-      </c>
-      <c r="C49" s="1" t="n">
-        <v>111.9139723976297</v>
-      </c>
-      <c r="D49" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E49" s="1" t="n">
-        <v>0.9774551240317242</v>
-      </c>
-      <c r="F49" s="1" t="n">
-        <v>1.012313512793219</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="inlineStr">
-        <is>
-          <t>Omnibus:</t>
-        </is>
-      </c>
-      <c r="B52" s="1" t="inlineStr">
-        <is>
-          <t>1180.145</t>
-        </is>
-      </c>
-      <c r="C52" s="1" t="inlineStr">
-        <is>
-          <t>Durbin-Watson:</t>
-        </is>
-      </c>
-      <c r="D52" s="1" t="inlineStr">
-        <is>
-          <t>1.648</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="inlineStr">
-        <is>
-          <t>Prob(Omnibus):</t>
-        </is>
-      </c>
-      <c r="B53" s="1" t="inlineStr">
-        <is>
-          <t>0.000</t>
-        </is>
-      </c>
-      <c r="C53" s="1" t="inlineStr">
-        <is>
-          <t>Jarque-Bera (JB):</t>
-        </is>
-      </c>
-      <c r="D53" s="1" t="inlineStr">
-        <is>
-          <t>22793.123</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="1" t="inlineStr">
-        <is>
-          <t>Skew:</t>
-        </is>
-      </c>
-      <c r="B54" s="1" t="inlineStr">
-        <is>
-          <t>1.001</t>
-        </is>
-      </c>
-      <c r="C54" s="1" t="inlineStr">
-        <is>
-          <t>Prob(JB):</t>
-        </is>
-      </c>
-      <c r="D54" s="1" t="inlineStr">
-        <is>
-          <t>0.000</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="1" t="inlineStr">
+      <c r="A48" s="1" t="inlineStr">
         <is>
           <t>Kurtosis:</t>
         </is>
       </c>
-      <c r="B55" s="1" t="inlineStr">
-        <is>
-          <t>14.885</t>
-        </is>
-      </c>
-      <c r="C55" s="1" t="inlineStr">
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>13.611</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
         <is>
           <t>Condition No.:</t>
         </is>
       </c>
-      <c r="D55" s="1" t="inlineStr">
-        <is>
-          <t>1888444098184045824</t>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>1491791</t>
         </is>
       </c>
     </row>

</xml_diff>